<commit_message>
feat: Add excel writer class.
</commit_message>
<xml_diff>
--- a/src/main/java/com/studyabroad/db/abroad_course_accounting_applications.xlsx
+++ b/src/main/java/com/studyabroad/db/abroad_course_accounting_applications.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
   <si>
     <t>University</t>
   </si>
@@ -61,12 +61,40 @@
   </si>
   <si>
     <t>Diplom</t>
+  </si>
+  <si>
+    <t>Humboldt University</t>
+  </si>
+  <si>
+    <t>Berlin</t>
+  </si>
+  <si>
+    <t>Germany</t>
+  </si>
+  <si>
+    <t>Introduction to Computer Science</t>
+  </si>
+  <si>
+    <t>https://www.informatik.hu-berlin.de/de/forschung/gebiete/algorithmenII/Lehre</t>
+  </si>
+  <si>
+    <t>Bachelor of Science</t>
+  </si>
+  <si>
+    <t>Pennsylvania University</t>
+  </si>
+  <si>
+    <t>Applied Econometrics</t>
+  </si>
+  <si>
+    <t>Master of Science</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
       <sz val="11"/>
@@ -412,13 +440,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="9.7109375"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="12.5703125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="12.140625"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="10.85546875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -450,6 +478,64 @@
         <v>8</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="n">
+        <v>232.0</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="n">
+        <v>12.0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>6.0</v>
+      </c>
+      <c r="H2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2345.0</v>
+      </c>
+      <c r="E3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1249.0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>6.0</v>
+      </c>
+      <c r="H3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I3" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Extend file with notes.
</commit_message>
<xml_diff>
--- a/src/main/java/com/studyabroad/db/abroad_course_accounting_applications.xlsx
+++ b/src/main/java/com/studyabroad/db/abroad_course_accounting_applications.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30215"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5737F066-DFD8-43D8-ACF3-F623DC4944A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FEC0AA55-E551-46A0-8E2E-533763CF1511}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -12,7 +12,7 @@
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>University</t>
   </si>
@@ -63,38 +63,13 @@
     <t>Diplom</t>
   </si>
   <si>
-    <t>Humboldt University</t>
-  </si>
-  <si>
-    <t>Berlin</t>
-  </si>
-  <si>
-    <t>Germany</t>
-  </si>
-  <si>
-    <t>Introduction to Computer Science</t>
-  </si>
-  <si>
-    <t>https://www.informatik.hu-berlin.de/de/forschung/gebiete/algorithmenII/Lehre</t>
-  </si>
-  <si>
-    <t>Bachelor of Science</t>
-  </si>
-  <si>
-    <t>Pennsylvania University</t>
-  </si>
-  <si>
-    <t>Applied Econometrics</t>
-  </si>
-  <si>
-    <t>Master of Science</t>
+    <t>Notes</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="1">
     <font>
       <sz val="11"/>
@@ -440,16 +415,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="9.7109375"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="12.5703125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="12.140625"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="10.85546875"/>
+    <col min="1" max="1" width="24.7109375" customWidth="1"/>
+    <col min="2" max="2" width="21.85546875" customWidth="1"/>
+    <col min="3" max="3" width="20.28515625" customWidth="1"/>
+    <col min="4" max="4" width="23.5703125" customWidth="1"/>
+    <col min="5" max="5" width="24.7109375" customWidth="1"/>
+    <col min="6" max="6" width="22.7109375" customWidth="1"/>
+    <col min="7" max="7" width="19.42578125" customWidth="1"/>
+    <col min="8" max="8" width="20.5703125" customWidth="1"/>
+    <col min="9" max="9" width="15.5703125" customWidth="1"/>
+    <col min="10" max="10" width="19.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:10">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -477,63 +458,8 @@
       <c r="I1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
+      <c r="J1" t="s">
         <v>9</v>
-      </c>
-      <c r="B2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" t="n">
-        <v>232.0</v>
-      </c>
-      <c r="E2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" t="n">
-        <v>12.0</v>
-      </c>
-      <c r="G2" t="n">
-        <v>6.0</v>
-      </c>
-      <c r="H2" t="s">
-        <v>13</v>
-      </c>
-      <c r="I2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" t="n">
-        <v>2345.0</v>
-      </c>
-      <c r="E3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" t="n">
-        <v>1249.0</v>
-      </c>
-      <c r="G3" t="n">
-        <v>6.0</v>
-      </c>
-      <c r="H3" t="s">
-        <v>13</v>
-      </c>
-      <c r="I3" t="s">
-        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: Add exception handling.
</commit_message>
<xml_diff>
--- a/src/main/java/com/studyabroad/db/abroad_course_accounting_applications.xlsx
+++ b/src/main/java/com/studyabroad/db/abroad_course_accounting_applications.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>University</t>
   </si>
@@ -64,12 +64,34 @@
   </si>
   <si>
     <t>Notes</t>
+  </si>
+  <si>
+    <t>Humboldt University</t>
+  </si>
+  <si>
+    <t>Berlin</t>
+  </si>
+  <si>
+    <t>Germany</t>
+  </si>
+  <si>
+    <t>Applied Econometrics</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>https://www.informatik.hu-berlin.de/de/forschung/gebiete/algorithmenII/Lehre</t>
+  </si>
+  <si>
+    <t>Master of Science</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
       <sz val="11"/>
@@ -415,19 +437,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="24.7109375" customWidth="1"/>
-    <col min="2" max="2" width="21.85546875" customWidth="1"/>
-    <col min="3" max="3" width="20.28515625" customWidth="1"/>
-    <col min="4" max="4" width="23.5703125" customWidth="1"/>
-    <col min="5" max="5" width="24.7109375" customWidth="1"/>
-    <col min="6" max="6" width="22.7109375" customWidth="1"/>
-    <col min="7" max="7" width="19.42578125" customWidth="1"/>
-    <col min="8" max="8" width="20.5703125" customWidth="1"/>
-    <col min="9" max="9" width="15.5703125" customWidth="1"/>
-    <col min="10" max="10" width="19.140625" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="24.7109375"/>
+    <col min="2" max="2" customWidth="true" width="21.85546875"/>
+    <col min="3" max="3" customWidth="true" width="20.28515625"/>
+    <col min="4" max="4" customWidth="true" width="23.5703125"/>
+    <col min="5" max="5" customWidth="true" width="24.7109375"/>
+    <col min="6" max="6" customWidth="true" width="22.7109375"/>
+    <col min="7" max="7" customWidth="true" width="19.42578125"/>
+    <col min="8" max="8" customWidth="true" width="20.5703125"/>
+    <col min="9" max="9" customWidth="true" width="15.5703125"/>
+    <col min="10" max="10" customWidth="true" width="19.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -462,6 +484,35 @@
         <v>9</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="n">
+        <v>12.0</v>
+      </c>
+      <c r="E2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" t="n">
+        <v>6.0</v>
+      </c>
+      <c r="H2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" t="s">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Add appropriate styling.
</commit_message>
<xml_diff>
--- a/src/main/java/com/studyabroad/db/abroad_course_accounting_applications.xlsx
+++ b/src/main/java/com/studyabroad/db/abroad_course_accounting_applications.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>University</t>
   </si>
@@ -64,34 +64,12 @@
   </si>
   <si>
     <t>Notes</t>
-  </si>
-  <si>
-    <t>Humboldt University</t>
-  </si>
-  <si>
-    <t>Berlin</t>
-  </si>
-  <si>
-    <t>Germany</t>
-  </si>
-  <si>
-    <t>Applied Econometrics</t>
-  </si>
-  <si>
-    <t>X</t>
-  </si>
-  <si>
-    <t>https://www.informatik.hu-berlin.de/de/forschung/gebiete/algorithmenII/Lehre</t>
-  </si>
-  <si>
-    <t>Master of Science</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="1">
     <font>
       <sz val="11"/>
@@ -437,19 +415,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="24.7109375"/>
-    <col min="2" max="2" customWidth="true" width="21.85546875"/>
-    <col min="3" max="3" customWidth="true" width="20.28515625"/>
-    <col min="4" max="4" customWidth="true" width="23.5703125"/>
-    <col min="5" max="5" customWidth="true" width="24.7109375"/>
-    <col min="6" max="6" customWidth="true" width="22.7109375"/>
-    <col min="7" max="7" customWidth="true" width="19.42578125"/>
-    <col min="8" max="8" customWidth="true" width="20.5703125"/>
-    <col min="9" max="9" customWidth="true" width="15.5703125"/>
-    <col min="10" max="10" customWidth="true" width="19.140625"/>
+    <col min="1" max="1" width="24.7109375" customWidth="1"/>
+    <col min="2" max="2" width="21.85546875" customWidth="1"/>
+    <col min="3" max="3" width="20.28515625" customWidth="1"/>
+    <col min="4" max="4" width="23.5703125" customWidth="1"/>
+    <col min="5" max="5" width="24.7109375" customWidth="1"/>
+    <col min="6" max="6" width="22.7109375" customWidth="1"/>
+    <col min="7" max="7" width="19.42578125" customWidth="1"/>
+    <col min="8" max="8" width="20.5703125" customWidth="1"/>
+    <col min="9" max="9" width="15.5703125" customWidth="1"/>
+    <col min="10" max="10" width="19.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -484,35 +462,6 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" t="n">
-        <v>12.0</v>
-      </c>
-      <c r="E2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" t="n">
-        <v>6.0</v>
-      </c>
-      <c r="H2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I2" t="s">
-        <v>16</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>